<commit_message>
Added a "Stop key" on Mono mode
</commit_message>
<xml_diff>
--- a/Fujiya Instruments/Junk Guitar/Junk Guitar/xlsx/VHG.xlsx
+++ b/Fujiya Instruments/Junk Guitar/Junk Guitar/xlsx/VHG.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="22730"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ADCEAFC-048B-4F4B-8F69-27E1D953B0EC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E173163-4FD6-4AFD-84AB-F295EE9CE687}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1320" yWindow="1005" windowWidth="25365" windowHeight="14160" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1110" yWindow="1140" windowWidth="25365" windowHeight="14160" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VHG Poly (Main)" sheetId="1" r:id="rId1"/>
@@ -1529,10 +1529,10 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1637,7 +1637,7 @@
     <xdr:to>
       <xdr:col>9</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>58</xdr:row>
+      <xdr:row>57</xdr:row>
       <xdr:rowOff>127000</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1950,7 +1950,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K132"/>
+  <dimension ref="A1:K131"/>
   <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="18.75"/>
   <cols>
     <col min="1" max="1" width="39.5" style="21" customWidth="1"/>
@@ -1964,7 +1964,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="24" t="s">
         <v>237</v>
       </c>
       <c r="B1" s="26" t="s">
@@ -2032,25 +2032,25 @@
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="1" t="s">
-        <v>250</v>
+        <v>143</v>
       </c>
       <c r="B5" s="19">
         <v>1</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>250</v>
-      </c>
-      <c r="D5" s="24" t="s">
+      <c r="C5" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D5" s="20" t="s">
         <v>12</v>
       </c>
       <c r="E5" s="19">
         <v>1</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="G5" s="19">
-        <v>15</v>
+        <v>120</v>
       </c>
       <c r="H5" s="19"/>
       <c r="I5" s="19"/>
@@ -2059,13 +2059,13 @@
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B6" s="19">
         <v>1</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D6" s="20" t="s">
         <v>12</v>
@@ -2074,7 +2074,7 @@
         <v>1</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G6" s="19">
         <v>120</v>
@@ -2086,13 +2086,13 @@
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B7" s="19">
         <v>1</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D7" s="20" t="s">
         <v>12</v>
@@ -2101,7 +2101,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G7" s="19">
         <v>120</v>
@@ -2113,13 +2113,13 @@
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B8" s="19">
         <v>1</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D8" s="20" t="s">
         <v>12</v>
@@ -2128,7 +2128,7 @@
         <v>1</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G8" s="19">
         <v>120</v>
@@ -2140,13 +2140,13 @@
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B9" s="19">
         <v>1</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D9" s="20" t="s">
         <v>12</v>
@@ -2155,7 +2155,7 @@
         <v>1</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G9" s="19">
         <v>120</v>
@@ -2167,13 +2167,13 @@
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B10" s="19">
         <v>1</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D10" s="20" t="s">
         <v>12</v>
@@ -2182,7 +2182,7 @@
         <v>1</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G10" s="19">
         <v>120</v>
@@ -2194,13 +2194,13 @@
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B11" s="19">
         <v>1</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D11" s="20" t="s">
         <v>12</v>
@@ -2209,7 +2209,7 @@
         <v>1</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G11" s="19">
         <v>120</v>
@@ -2221,13 +2221,13 @@
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B12" s="19">
         <v>1</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D12" s="20" t="s">
         <v>12</v>
@@ -2236,7 +2236,7 @@
         <v>1</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G12" s="19">
         <v>120</v>
@@ -2248,13 +2248,13 @@
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B13" s="19">
         <v>1</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D13" s="20" t="s">
         <v>12</v>
@@ -2263,7 +2263,7 @@
         <v>1</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G13" s="19">
         <v>120</v>
@@ -2275,13 +2275,13 @@
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B14" s="19">
         <v>1</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D14" s="20" t="s">
         <v>12</v>
@@ -2290,7 +2290,7 @@
         <v>1</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G14" s="19">
         <v>120</v>
@@ -2302,13 +2302,13 @@
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B15" s="19">
         <v>1</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D15" s="20" t="s">
         <v>12</v>
@@ -2317,7 +2317,7 @@
         <v>1</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G15" s="19">
         <v>120</v>
@@ -2329,13 +2329,13 @@
     </row>
     <row r="16" spans="1:11">
       <c r="A16" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B16" s="19">
         <v>1</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D16" s="20" t="s">
         <v>12</v>
@@ -2344,7 +2344,7 @@
         <v>1</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G16" s="19">
         <v>120</v>
@@ -2356,13 +2356,13 @@
     </row>
     <row r="17" spans="1:11">
       <c r="A17" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B17" s="19">
         <v>1</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D17" s="20" t="s">
         <v>12</v>
@@ -2371,7 +2371,7 @@
         <v>1</v>
       </c>
       <c r="F17" s="19" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G17" s="19">
         <v>120</v>
@@ -2383,13 +2383,13 @@
     </row>
     <row r="18" spans="1:11">
       <c r="A18" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B18" s="19">
         <v>1</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D18" s="20" t="s">
         <v>12</v>
@@ -2398,7 +2398,7 @@
         <v>1</v>
       </c>
       <c r="F18" s="19" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G18" s="19">
         <v>120</v>
@@ -2410,13 +2410,13 @@
     </row>
     <row r="19" spans="1:11">
       <c r="A19" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B19" s="19">
         <v>1</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D19" s="20" t="s">
         <v>12</v>
@@ -2425,7 +2425,7 @@
         <v>1</v>
       </c>
       <c r="F19" s="19" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G19" s="19">
         <v>120</v>
@@ -2437,13 +2437,13 @@
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B20" s="19">
         <v>1</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D20" s="20" t="s">
         <v>12</v>
@@ -2452,7 +2452,7 @@
         <v>1</v>
       </c>
       <c r="F20" s="19" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G20" s="19">
         <v>120</v>
@@ -2463,27 +2463,13 @@
       <c r="K20" s="19"/>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="B21" s="19">
-        <v>1</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="D21" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="E21" s="19">
-        <v>1</v>
-      </c>
-      <c r="F21" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="G21" s="19">
-        <v>120</v>
-      </c>
+      <c r="A21" s="1"/>
+      <c r="B21" s="19"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="19"/>
+      <c r="F21" s="19"/>
+      <c r="G21" s="19"/>
       <c r="H21" s="19"/>
       <c r="I21" s="19"/>
       <c r="J21" s="19"/>
@@ -3919,42 +3905,29 @@
       <c r="J131" s="19"/>
       <c r="K131" s="19"/>
     </row>
-    <row r="132" spans="1:11">
-      <c r="A132" s="1"/>
-      <c r="B132" s="19"/>
-      <c r="C132" s="2"/>
-      <c r="D132" s="20"/>
-      <c r="E132" s="19"/>
-      <c r="F132" s="19"/>
-      <c r="G132" s="19"/>
-      <c r="H132" s="19"/>
-      <c r="I132" s="19"/>
-      <c r="J132" s="19"/>
-      <c r="K132" s="19"/>
-    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B1:C1"/>
   </mergeCells>
   <phoneticPr fontId="7"/>
   <dataValidations count="5">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B4:B132" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B4:B131" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"0,1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="0-127" prompt="If don't use CC set cell value empty" sqref="H4:I132" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="0-127" prompt="If don't use CC set cell value empty" sqref="H4:I131" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>0</formula1>
       <formula2>127</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="0-127" prompt="If don't use MIDI Note on, set cell value empty." sqref="G4:G132" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="0-127" prompt="If don't use MIDI Note on, set cell value empty." sqref="G4:G131" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>0</formula1>
       <formula2>127</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="0-127" prompt="If don't use Program Change, set cell value empty." sqref="J4:J132" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="0-127" prompt="If don't use Program Change, set cell value empty." sqref="J4:J131" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>0</formula1>
       <formula2>127</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="0-127" prompt="If cell value is empty, MSB will be set 0._x000a__x000a_By my research, Maybe Cubase will not recognize MSB." sqref="K4:K132" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="0-127" prompt="If cell value is empty, MSB will be set 0._x000a__x000a_By my research, Maybe Cubase will not recognize MSB." sqref="K4:K131" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>0</formula1>
       <formula2>127</formula2>
     </dataValidation>
@@ -3973,7 +3946,7 @@
           <x14:formula2>
             <xm:f>0</xm:f>
           </x14:formula2>
-          <xm:sqref>D4:D132</xm:sqref>
+          <xm:sqref>D4:D131</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000006000000}">
           <x14:formula1>
@@ -3982,7 +3955,7 @@
           <x14:formula2>
             <xm:f>0</xm:f>
           </x14:formula2>
-          <xm:sqref>E4:E132</xm:sqref>
+          <xm:sqref>E4:E131</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" showInputMessage="1" showErrorMessage="1" promptTitle="MIDI Note" prompt="Choose from Drop-down list or imput number directly(0-127)_x000a__x000a_If don’t use MIDI Note, set Cell value empty." xr:uid="{00000000-0002-0000-0000-000007000000}">
           <x14:formula1>
@@ -3991,7 +3964,7 @@
           <x14:formula2>
             <xm:f>0</xm:f>
           </x14:formula2>
-          <xm:sqref>F4:F132</xm:sqref>
+          <xm:sqref>F4:F131</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -4015,7 +3988,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="24" t="s">
         <v>237</v>
       </c>
       <c r="B1" s="26" t="s">
@@ -5996,7 +5969,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="24" t="s">
         <v>237</v>
       </c>
       <c r="B1" s="26" t="s">
@@ -7837,7 +7810,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="24" t="s">
         <v>237</v>
       </c>
       <c r="B1" s="26" t="s">
@@ -11320,7 +11293,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="24" t="s">
         <v>237</v>
       </c>
       <c r="B1" s="26" t="s">
@@ -13177,7 +13150,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:K131"/>
+  <dimension ref="A1:K132"/>
   <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="18.75"/>
   <cols>
     <col min="1" max="1" width="39.5" style="21" customWidth="1"/>
@@ -13191,7 +13164,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="24" t="s">
         <v>237</v>
       </c>
       <c r="B1" s="26" t="s">
@@ -13259,25 +13232,25 @@
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="1" t="s">
-        <v>164</v>
+        <v>250</v>
       </c>
       <c r="B5" s="19">
         <v>1</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="D5" s="20" t="s">
+      <c r="C5" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="D5" s="25" t="s">
         <v>12</v>
       </c>
       <c r="E5" s="19">
         <v>1</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="G5" s="19">
-        <v>120</v>
+        <v>15</v>
       </c>
       <c r="H5" s="19"/>
       <c r="I5" s="19"/>
@@ -13286,13 +13259,13 @@
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B6" s="19">
         <v>1</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D6" s="20" t="s">
         <v>12</v>
@@ -13301,7 +13274,7 @@
         <v>1</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G6" s="19">
         <v>120</v>
@@ -13313,13 +13286,13 @@
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B7" s="19">
         <v>1</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D7" s="20" t="s">
         <v>12</v>
@@ -13328,7 +13301,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G7" s="19">
         <v>120</v>
@@ -13340,13 +13313,13 @@
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B8" s="19">
         <v>1</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D8" s="20" t="s">
         <v>12</v>
@@ -13355,7 +13328,7 @@
         <v>1</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G8" s="19">
         <v>120</v>
@@ -13367,13 +13340,13 @@
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B9" s="19">
         <v>1</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D9" s="20" t="s">
         <v>12</v>
@@ -13382,7 +13355,7 @@
         <v>1</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G9" s="19">
         <v>120</v>
@@ -13394,13 +13367,13 @@
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="1" t="s">
-        <v>145</v>
+        <v>168</v>
       </c>
       <c r="B10" s="19">
         <v>1</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>145</v>
+        <v>168</v>
       </c>
       <c r="D10" s="20" t="s">
         <v>12</v>
@@ -13409,7 +13382,7 @@
         <v>1</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G10" s="19">
         <v>120</v>
@@ -13421,13 +13394,13 @@
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B11" s="19">
         <v>1</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D11" s="20" t="s">
         <v>12</v>
@@ -13436,7 +13409,7 @@
         <v>1</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G11" s="19">
         <v>120</v>
@@ -13448,13 +13421,13 @@
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B12" s="19">
         <v>1</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D12" s="20" t="s">
         <v>12</v>
@@ -13463,7 +13436,7 @@
         <v>1</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G12" s="19">
         <v>120</v>
@@ -13475,13 +13448,13 @@
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B13" s="19">
         <v>1</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D13" s="20" t="s">
         <v>12</v>
@@ -13490,7 +13463,7 @@
         <v>1</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G13" s="19">
         <v>120</v>
@@ -13502,13 +13475,13 @@
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B14" s="19">
         <v>1</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D14" s="20" t="s">
         <v>12</v>
@@ -13517,7 +13490,7 @@
         <v>1</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G14" s="19">
         <v>120</v>
@@ -13529,13 +13502,13 @@
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B15" s="19">
         <v>1</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D15" s="20" t="s">
         <v>12</v>
@@ -13544,7 +13517,7 @@
         <v>1</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G15" s="19">
         <v>120</v>
@@ -13556,13 +13529,13 @@
     </row>
     <row r="16" spans="1:11">
       <c r="A16" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B16" s="19">
         <v>1</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D16" s="20" t="s">
         <v>12</v>
@@ -13571,7 +13544,7 @@
         <v>1</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G16" s="19">
         <v>120</v>
@@ -13583,13 +13556,13 @@
     </row>
     <row r="17" spans="1:11">
       <c r="A17" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B17" s="19">
         <v>1</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D17" s="20" t="s">
         <v>12</v>
@@ -13598,7 +13571,7 @@
         <v>1</v>
       </c>
       <c r="F17" s="19" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G17" s="19">
         <v>120</v>
@@ -13610,13 +13583,13 @@
     </row>
     <row r="18" spans="1:11">
       <c r="A18" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B18" s="19">
         <v>1</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D18" s="20" t="s">
         <v>12</v>
@@ -13625,7 +13598,7 @@
         <v>1</v>
       </c>
       <c r="F18" s="19" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G18" s="19">
         <v>120</v>
@@ -13637,13 +13610,13 @@
     </row>
     <row r="19" spans="1:11">
       <c r="A19" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B19" s="19">
         <v>1</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D19" s="20" t="s">
         <v>12</v>
@@ -13652,7 +13625,7 @@
         <v>1</v>
       </c>
       <c r="F19" s="19" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G19" s="19">
         <v>120</v>
@@ -13664,13 +13637,13 @@
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="1" t="s">
-        <v>169</v>
+        <v>154</v>
       </c>
       <c r="B20" s="19">
         <v>1</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>169</v>
+        <v>154</v>
       </c>
       <c r="D20" s="20" t="s">
         <v>12</v>
@@ -13679,7 +13652,7 @@
         <v>1</v>
       </c>
       <c r="F20" s="19" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G20" s="19">
         <v>120</v>
@@ -13691,13 +13664,13 @@
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B21" s="19">
         <v>1</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D21" s="20" t="s">
         <v>12</v>
@@ -13706,7 +13679,7 @@
         <v>1</v>
       </c>
       <c r="F21" s="19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G21" s="19">
         <v>120</v>
@@ -13718,13 +13691,13 @@
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="1" t="s">
-        <v>156</v>
+        <v>170</v>
       </c>
       <c r="B22" s="19">
         <v>1</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>156</v>
+        <v>170</v>
       </c>
       <c r="D22" s="20" t="s">
         <v>12</v>
@@ -13733,7 +13706,7 @@
         <v>1</v>
       </c>
       <c r="F22" s="19" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G22" s="19">
         <v>120</v>
@@ -13745,13 +13718,13 @@
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B23" s="19">
         <v>1</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D23" s="20" t="s">
         <v>12</v>
@@ -13760,7 +13733,7 @@
         <v>1</v>
       </c>
       <c r="F23" s="19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G23" s="19">
         <v>120</v>
@@ -13772,13 +13745,13 @@
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B24" s="19">
         <v>1</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D24" s="20" t="s">
         <v>12</v>
@@ -13787,7 +13760,7 @@
         <v>1</v>
       </c>
       <c r="F24" s="19" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G24" s="19">
         <v>120</v>
@@ -13798,13 +13771,27 @@
       <c r="K24" s="19"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="1"/>
-      <c r="B25" s="19"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="20"/>
-      <c r="E25" s="19"/>
-      <c r="F25" s="19"/>
-      <c r="G25" s="19"/>
+      <c r="A25" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="B25" s="19">
+        <v>1</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="D25" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" s="19">
+        <v>1</v>
+      </c>
+      <c r="F25" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="G25" s="19">
+        <v>120</v>
+      </c>
       <c r="H25" s="19"/>
       <c r="I25" s="19"/>
       <c r="J25" s="19"/>
@@ -15188,29 +15175,42 @@
       <c r="J131" s="19"/>
       <c r="K131" s="19"/>
     </row>
+    <row r="132" spans="1:11">
+      <c r="A132" s="1"/>
+      <c r="B132" s="19"/>
+      <c r="C132" s="2"/>
+      <c r="D132" s="20"/>
+      <c r="E132" s="19"/>
+      <c r="F132" s="19"/>
+      <c r="G132" s="19"/>
+      <c r="H132" s="19"/>
+      <c r="I132" s="19"/>
+      <c r="J132" s="19"/>
+      <c r="K132" s="19"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B1:C1"/>
   </mergeCells>
   <phoneticPr fontId="8"/>
   <dataValidations count="5">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B4:B131" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B4:B132" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"0,1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="0-127" prompt="If don't use CC set cell value empty" sqref="H4:I131" xr:uid="{00000000-0002-0000-0200-000001000000}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="0-127" prompt="If don't use CC set cell value empty" sqref="H4:I132" xr:uid="{00000000-0002-0000-0200-000001000000}">
       <formula1>0</formula1>
       <formula2>127</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="0-127" prompt="If don't use MIDI Note on, set cell value empty." sqref="G4:G131" xr:uid="{00000000-0002-0000-0200-000002000000}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="0-127" prompt="If don't use MIDI Note on, set cell value empty." sqref="G4:G132" xr:uid="{00000000-0002-0000-0200-000002000000}">
       <formula1>0</formula1>
       <formula2>127</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="0-127" prompt="If don't use Program Change, set cell value empty." sqref="J4:J131" xr:uid="{00000000-0002-0000-0200-000003000000}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="0-127" prompt="If don't use Program Change, set cell value empty." sqref="J4:J132" xr:uid="{00000000-0002-0000-0200-000003000000}">
       <formula1>0</formula1>
       <formula2>127</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="0-127" prompt="If cell value is empty, MSB will be set 0._x000a__x000a_By my research, Maybe Cubase will not recognize MSB." sqref="K4:K131" xr:uid="{00000000-0002-0000-0200-000004000000}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="0-127" prompt="If cell value is empty, MSB will be set 0._x000a__x000a_By my research, Maybe Cubase will not recognize MSB." sqref="K4:K132" xr:uid="{00000000-0002-0000-0200-000004000000}">
       <formula1>0</formula1>
       <formula2>127</formula2>
     </dataValidation>
@@ -15228,7 +15228,7 @@
           <x14:formula2>
             <xm:f>0</xm:f>
           </x14:formula2>
-          <xm:sqref>D4:D131</xm:sqref>
+          <xm:sqref>D4:D132</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000006000000}">
           <x14:formula1>
@@ -15237,7 +15237,7 @@
           <x14:formula2>
             <xm:f>0</xm:f>
           </x14:formula2>
-          <xm:sqref>E4:E131</xm:sqref>
+          <xm:sqref>E4:E132</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" showInputMessage="1" showErrorMessage="1" promptTitle="MIDI Note" prompt="Choose from Drop-down list or imput number directly(0-127)_x000a__x000a_If don’t use MIDI Note, set Cell value empty." xr:uid="{00000000-0002-0000-0200-000007000000}">
           <x14:formula1>
@@ -15246,7 +15246,7 @@
           <x14:formula2>
             <xm:f>0</xm:f>
           </x14:formula2>
-          <xm:sqref>F4:F131</xm:sqref>
+          <xm:sqref>F4:F132</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -15270,7 +15270,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="24" t="s">
         <v>237</v>
       </c>
       <c r="B1" s="26" t="s">
@@ -17111,7 +17111,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="24" t="s">
         <v>237</v>
       </c>
       <c r="B1" s="26" t="s">
@@ -19134,7 +19134,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="24" t="s">
         <v>237</v>
       </c>
       <c r="B1" s="26" t="s">
@@ -21269,7 +21269,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="24" t="s">
         <v>237</v>
       </c>
       <c r="B1" s="26" t="s">
@@ -23124,7 +23124,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="24" t="s">
         <v>237</v>
       </c>
       <c r="B1" s="26" t="s">
@@ -24951,7 +24951,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="24" t="s">
         <v>237</v>
       </c>
       <c r="B1" s="26" t="s">

</xml_diff>